<commit_message>
feat: save accepted 0.5G ballistics and client fixes with configuration guards
</commit_message>
<xml_diff>
--- a/docs/RTT_GAME_DATA.xlsx
+++ b/docs/RTT_GAME_DATA.xlsx
@@ -1904,8 +1904,8 @@
       <x:c r="H15" s="4" t="str">
         <x:v>不适用</x:v>
       </x:c>
-      <x:c r="I15" s="4" t="n">
-        <x:v>810</x:v>
+      <x:c r="I15" s="4" t="str">
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="J15" s="4" t="n">
         <x:v>8</x:v>

</xml_diff>